<commit_message>
06/09/2026, 07/09/2026, 09/09/2026, 10/09/2026 AU
</commit_message>
<xml_diff>
--- a/12612645.xlsx
+++ b/12612645.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shash\Desktop\Activities\12612645\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EF9565-E71C-49C1-B4C5-DAB719C7C7F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5BA531-34FC-4AFB-A14F-5FEDB54C8A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1930,158 +1930,312 @@
       </c>
       <c r="N25" s="17"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+    <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="8">
+        <v>46271</v>
+      </c>
+      <c r="B26" s="14">
+        <v>480</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="14">
+        <v>360</v>
+      </c>
+      <c r="E26" s="14">
+        <v>240</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14">
+        <v>300</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1380</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
+        <v>60</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+      <c r="A27" s="8">
+        <v>46272</v>
+      </c>
+      <c r="B27" s="14">
+        <v>240</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="14">
+        <v>180</v>
+      </c>
+      <c r="E27" s="14">
+        <v>180</v>
+      </c>
+      <c r="F27" s="14">
+        <v>200</v>
+      </c>
+      <c r="G27" s="14">
+        <v>4</v>
+      </c>
+      <c r="H27" s="14">
+        <v>240</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="8">
+        <v>46273</v>
+      </c>
+      <c r="B28" s="14">
+        <v>180</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="14">
+        <v>240</v>
+      </c>
+      <c r="E28" s="14">
+        <v>90</v>
+      </c>
+      <c r="F28" s="14">
+        <v>300</v>
+      </c>
+      <c r="G28" s="14">
+        <v>6</v>
+      </c>
+      <c r="H28" s="14">
+        <v>180</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+        <v>450</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="8">
+        <v>46274</v>
+      </c>
+      <c r="B29" s="14">
+        <v>210</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="14">
+        <v>180</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>350</v>
+      </c>
+      <c r="G29" s="14">
+        <v>7</v>
+      </c>
+      <c r="H29" s="14">
+        <v>240</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
+        <v>460</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N29" s="17"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+    <row r="30" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="8">
+        <v>46275</v>
+      </c>
+      <c r="B30" s="14">
+        <v>240</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="14">
+        <v>240</v>
+      </c>
+      <c r="E30" s="14">
+        <v>180</v>
+      </c>
+      <c r="F30" s="14">
+        <v>200</v>
+      </c>
+      <c r="G30" s="14">
+        <v>4</v>
+      </c>
+      <c r="H30" s="14">
+        <v>180</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N30" s="17"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="8">
+        <v>46276</v>
+      </c>
+      <c r="B31" s="14">
+        <v>180</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="14">
+        <v>300</v>
+      </c>
+      <c r="E31" s="14">
+        <v>120</v>
+      </c>
+      <c r="F31" s="14">
+        <v>250</v>
+      </c>
+      <c r="G31" s="14">
+        <v>5</v>
+      </c>
+      <c r="H31" s="14">
+        <v>210</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
+        <v>380</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N31" s="17"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+      <c r="A32" s="8">
+        <v>46277</v>
+      </c>
+      <c r="B32" s="14">
+        <v>480</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="14">
+        <v>240</v>
+      </c>
+      <c r="E32" s="14">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14">
+        <v>0</v>
+      </c>
+      <c r="G32" s="14">
+        <v>0</v>
+      </c>
+      <c r="H32" s="14">
+        <v>240</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
+        <v>480</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N32" s="17"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
11/09/2026 and 12/09/2026 Activity update.
</commit_message>
<xml_diff>
--- a/12612645.xlsx
+++ b/12612645.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shash\Desktop\Activities\12612645\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5BA531-34FC-4AFB-A14F-5FEDB54C8A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C23A2D8-634E-443C-961E-232199AF1CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2231,7 +2231,7 @@
         <v>62</v>
       </c>
       <c r="L32" s="16" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="M32" s="16" t="s">
         <v>60</v>

</xml_diff>